<commit_message>
F-BS3: the Ltd corporation tax charge and the interest tax credit round to pence
Engine and template carried the marginal-relief charge unrounded, and the CT600
boxes recomputed it from unrounded rows, so tax payable, the trial balance
creditor and the published balance sheet were fractions of a penny. The charge
now rounds at CorporationTax!K35 (CT600 box 65 reads K35), and the grossed-up
interest tax credit rounds at its source, TrialBalance!EH58, in both engine and
template, so K37, K39, CT600 box 84 and EJ35 follow in pence with no balancing
adjustment. Ltd parity fixture and examples/ltd-latest regenerated; reconcile
1103/1103, equivalence spec 10/10, parity.sh all four products match.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-sonnet-5-5
Claude-Session: https://claude.ai/code/session_01HncMnj3gY1YfX4FmQC3Ki2
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Financialaccounts.xlsx
+++ b/app/templates/ltd/Financialaccounts.xlsx
@@ -30694,7 +30694,7 @@
       </c>
       <c r="EG58" s="13"/>
       <c r="EH58" s="22">
-        <f>IF(OpenAccounts!P8="X",0,EF58/((100-Admin!P7)/100)-EF58)</f>
+        <f>ROUND(IF(OpenAccounts!P8="X",0,EF58/((100-Admin!P7)/100)-EF58),2)</f>
         <v>0</v>
       </c>
       <c r="EI58" s="13"/>
@@ -45203,7 +45203,7 @@
       <c r="I35" s="188"/>
       <c r="J35" s="188"/>
       <c r="K35" s="189">
-        <f>SUM(I33:I34)</f>
+        <f>ROUND(SUM(I33:I34),2)</f>
         <v>0</v>
       </c>
       <c r="L35" s="39"/>
@@ -53434,7 +53434,7 @@
       </c>
       <c r="X135" s="225"/>
       <c r="Y135" s="535">
-        <f>AJ131-Y133</f>
+        <f>CorporationTax!K35</f>
         <v>0</v>
       </c>
       <c r="Z135" s="535"/>

</xml_diff>